<commit_message>
📊 Daily DSE update
</commit_message>
<xml_diff>
--- a/dse_market_summary.xlsx
+++ b/dse_market_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Market Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I471"/>
+  <dimension ref="A1:I472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22581,6 +22581,53 @@
         </is>
       </c>
     </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>180,803,676</t>
+        </is>
+      </c>
+      <c r="B472" s="2" t="inlineStr">
+        <is>
+          <t>1,954.44755</t>
+        </is>
+      </c>
+      <c r="C472" s="2" t="inlineStr">
+        <is>
+          <t>Apr 06, 2026</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>5,122.53162</t>
+        </is>
+      </c>
+      <c r="E472" s="2" t="inlineStr">
+        <is>
+          <t>9.10865</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="inlineStr">
+        <is>
+          <t>10.26091</t>
+        </is>
+      </c>
+      <c r="G472" s="2" t="inlineStr">
+        <is>
+          <t>4,707.925</t>
+        </is>
+      </c>
+      <c r="H472" s="2" t="inlineStr">
+        <is>
+          <t>6,812,534.040</t>
+        </is>
+      </c>
+      <c r="I472" s="2" t="inlineStr">
+        <is>
+          <t>149,305</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>